<commit_message>
Fix forced alignment sample audio
</commit_message>
<xml_diff>
--- a/sample_data/speech_annotator_test_upload.xlsx
+++ b/sample_data/speech_annotator_test_upload.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="annotation_tasks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="annotation_tasks" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>4.2</v>
+        <v>9.807</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>3.7</v>
+        <v>5.933</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>4.8</v>
+        <v>6.258</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>3.9</v>
+        <v>7.327</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>3.4</v>
+        <v>6.897</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>5.1</v>
+        <v>6.541</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>3.6</v>
+        <v>5.467</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1153,7 +1153,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>4.4</v>
+        <v>10.914</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>4</v>
+        <v>3.785</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>4.6</v>
+        <v>6.325</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>

</xml_diff>